<commit_message>
Enter remaining dry10 headers after parse teach, including Orthman 9931.
SpectrumVoIP 929030 stays Fail (vendor missing on live). Cursor unchanged.
Headers 9921-9931 on batch 701 still need live UI Select Receipts + PDF.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-08-dry10.xlsx
+++ b/runs/AP-run-2026-09-08-dry10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="AP run" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$O$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AP run'!$A$1:$O$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -692,7 +692,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Cecilia Hulsey</t>
+          <t>Orthman Conveying Systems</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -713,17 +713,19 @@
       <c r="E4" s="2" t="n">
         <v>1242.94</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Fail: vendor missing on live for Cecilia Hulsey (PO 58636 exists as PO58636-Orthman Conveying). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>Incomplete (finish): header created (id 9931). Select Receipts not posted (API not Editable; live UI path required). Do not type Add Item. PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Attach status=blocked-405. Flag status=ai-hold.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>9931</v>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/8/26 (701)</t>
@@ -741,7 +743,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -824,34 +826,40 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>RMP Industrial Supply Inc</t>
+          <t>Fastenal Company</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1471255</t>
+          <t>TXFT499945</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>58841</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="n">
-        <v>67.48999999999999</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>62.98</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD parse-error (preflight-parse): invoice # must be taken from vendor PDF text, not email subject/filename alone (MSC/McQueary). Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>Incomplete (finish): header created (id 9930). Select Receipts not posted (API not Editable; live UI path required). Do not type Add Item. PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Attach status=blocked-405. Flag status=ai-hold.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>9930</v>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/8/26 (701)</t>
@@ -859,7 +867,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Shipping &amp; Handling 15.31</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -869,7 +877,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -887,12 +895,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>UniFirst Corporation</t>
+          <t>RMP Industrial Supply Inc</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2810795106</t>
+          <t>1471255</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -900,25 +908,23 @@
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>58002</t>
-        </is>
-      </c>
+      <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="n">
-        <v>1333.48</v>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>67.48999999999999</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HOLD parse-error (preflight-parse): invoice # must be taken from vendor PDF text, not email subject/filename alone (MSC/McQueary). Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
+          <t>Incomplete (finish): header created (id 9927). PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Purchase Order left blank (no-PO or multi-PO). Do not type Add Item. Attach status=blocked-405. Flag status=ai-hold.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>9927</v>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/8/26 (701)</t>
@@ -926,7 +932,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>3.00Energy Surcharge 0.25 3.25ENER 3.0000 3.00; 7.0492.21 99.25885 Garment Maintenance Protection (GMP) 99.25; 2.9835.40 38.38885 Garment Setup Protection (GSP) 38.38; 7.3887.51 94.89885 Garment Loss Protection (GLP) 94.89; 2.2428.26 30.50471 Garment Emblem Protection (GEP) 30.50</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -936,7 +942,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -954,12 +960,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Air Products and Chemicals, Inc</t>
+          <t>UniFirst Corporation</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>436150428</t>
+          <t>2810795106</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -969,7 +975,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="n">
-        <v>1299</v>
+        <v>1333.48</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
@@ -978,11 +984,11 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Incomplete (finish): header created (id 9925). PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Purchase Order left blank (no-PO or multi-PO). Do not type Add Item. Attach status=blocked-405. Flag status=ai-hold.</t>
+          <t>Incomplete (finish): header created (id 9928). PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Purchase Order left blank (no-PO or multi-PO). Do not type Add Item. Attach status=blocked-405. Flag status=ai-hold.</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>9925</v>
+        <v>9928</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -991,7 +997,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>3.00Energy Surcharge 0.25 3.25ENER 3.0000 3.00; 7.0492.21 99.25885 Garment Maintenance Protection (GMP) 99.25; 2.9835.40 38.38885 Garment Setup Protection (GSP) 38.38; 7.3887.51 94.89885 Garment Loss Protection (GLP) 94.89; 2.2428.26 30.50471 Garment Emblem Protection (GEP) 30.50</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1019,12 +1025,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Earle M. Jorgensen Co</t>
+          <t>Air Products and Chemicals, Inc</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>S813828432</t>
+          <t>436150428</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1032,13 +1038,9 @@
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>58927</t>
-        </is>
-      </c>
+      <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="n">
-        <v>421.2</v>
+        <v>1299</v>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
@@ -1047,11 +1049,11 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Incomplete (finish): header created (id 9926). Select Receipts not posted (API not Editable; live UI path required). Do not type Add Item. PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Attach status=blocked-405. Flag status=ai-hold.</t>
+          <t>Incomplete (finish): header created (id 9925). PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Purchase Order left blank (no-PO or multi-PO). Do not type Add Item. Attach status=blocked-405. Flag status=ai-hold.</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>9926</v>
+        <v>9925</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1062,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>SHIPPING DATE 14-AUG-2026; FREIGHT PAYMENT PREPAID</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1088,30 +1090,40 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PCT Support</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr"/>
+          <t>Earle M. Jorgensen Co</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>S813828432</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>58927</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="n">
-        <v>1310</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>421.2</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>HOLD parse-error (preflight-parse): invoice # must be taken from vendor PDF text, not email subject/filename alone (MSC/McQueary). Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
+          <t>Incomplete (finish): header created (id 9926). Select Receipts not posted (API not Editable; live UI path required). Do not type Add Item. PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Header PO set. Select Receipts via API not implemented without an Editable receipt action; do not type Add Item. Select Receipts: 1 receipt(s) matched by part/PO-WO/slip (not first qty). Attach status=blocked-405. Flag status=ai-hold.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>9926</v>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/8/26 (701)</t>
@@ -1119,7 +1131,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>SHIPPING DATE 14-AUG-2026; FREIGHT PAYMENT PREPAID</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1129,7 +1141,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1147,34 +1159,36 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SpectrumVoIP Billing</t>
+          <t>PCT Support</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>929030</t>
+          <t>LS-8507</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="n">
-        <v>33.39</v>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+        <v>1310</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>HOLD parse-error (preflight-parse): invoice # must be taken from vendor PDF text, not email subject/filename alone (MSC/McQueary). Flag status=ai-hold.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+          <t>Incomplete (finish): header created (id 9929). PDF attach=blocked-405. Success requires the vendor PDF on the header. Not Entered in AI. Purchase Order left blank (no-PO or multi-PO). Do not type Add Item. Attach status=blocked-405. Flag status=ai-hold.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>9929</v>
+      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>API Agent - 9/8/26 (701)</t>
@@ -1182,7 +1196,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Taxes and Surcharges 9.41; FEDERAL COST RECOVERY FEE .46</t>
+          <t>none</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1192,7 +1206,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>no-pdf-on-vm</t>
+          <t>blocked-405</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1210,36 +1224,42 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Globe Life</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr"/>
+          <t>SpectrumVoIP</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>929030</t>
+        </is>
+      </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="E12" s="2" t="n">
+        <v>33.39</v>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>HOLD (bill-vs-noise): not-a-bill. Do not create a header. Flag status=ai-hold.</t>
+          <t>Fail: vendor missing on live for SpectrumVoIP (looked up by vendor name / alias / PO vendor). Will not invent a vendor/remit-to ID. Flag status=ai-hold.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>API Agent - 9/8/26</t>
+          <t>API Agent - 9/8/26 (701)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Taxes and Surcharges 9.41; FEDERAL COST RECOVERY FEE .46</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1321,8 +1341,65 @@
       </c>
       <c r="O13" s="2" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Globe Life</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>HOLD (bill-vs-noise): not-a-bill. Do not create a header. Flag status=ai-hold.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>API Agent - 9/8/26</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>no-pdf-on-vm</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>ai-hold</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O13"/>
+  <autoFilter ref="A1:O14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>